<commit_message>
Alterações na geração da planilha
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -11,7 +11,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="16">
+  <si>
+    <t>Candidatos</t>
+  </si>
   <si>
     <t>Nome</t>
   </si>
@@ -28,6 +31,9 @@
     <t>Sexo</t>
   </si>
   <si>
+    <t>Tipo</t>
+  </si>
+  <si>
     <t>teste</t>
   </si>
   <si>
@@ -41,6 +47,18 @@
   </si>
   <si>
     <t>Masculino</t>
+  </si>
+  <si>
+    <t>mestrado</t>
+  </si>
+  <si>
+    <t>Professores</t>
+  </si>
+  <si>
+    <t>teste2</t>
+  </si>
+  <si>
+    <t>doutorado</t>
   </si>
 </sst>
 </file>
@@ -56,12 +74,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FFC0C0C0"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -76,8 +100,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,47 +447,123 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="5" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C3" t="s">
         <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modificações no estilo das linhas.
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -4,74 +4,83 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Planilha de Candidatos" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Candidato" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Provas" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Propostas" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="16">
-  <si>
-    <t>Candidatos</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="16">
+  <si>
+    <t>Mestrados</t>
   </si>
   <si>
     <t>Nome</t>
   </si>
   <si>
-    <t>CPF</t>
-  </si>
-  <si>
-    <t>RG</t>
-  </si>
-  <si>
-    <t>Data de Nascimento</t>
-  </si>
-  <si>
-    <t>Sexo</t>
-  </si>
-  <si>
-    <t>Tipo</t>
-  </si>
-  <si>
-    <t>teste</t>
-  </si>
-  <si>
-    <t>12345678910</t>
-  </si>
-  <si>
-    <t>123456789</t>
-  </si>
-  <si>
-    <t>01/01/2000</t>
-  </si>
-  <si>
-    <t>Masculino</t>
-  </si>
-  <si>
-    <t>mestrado</t>
-  </si>
-  <si>
-    <t>Professores</t>
-  </si>
-  <si>
-    <t>teste2</t>
-  </si>
-  <si>
-    <t>doutorado</t>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Inscrição</t>
+  </si>
+  <si>
+    <t>Linha</t>
+  </si>
+  <si>
+    <t>Orientador</t>
+  </si>
+  <si>
+    <t>Bolsa</t>
+  </si>
+  <si>
+    <t>Nível</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>asd@email.com</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Doutorados</t>
+  </si>
+  <si>
+    <t>{"header":"Nome","key":"nome","width":30}</t>
+  </si>
+  <si>
+    <t>Teste2</t>
+  </si>
+  <si>
+    <t>asd@asd.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="00000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -100,12 +109,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,127 +457,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="6" width="10" customWidth="1"/>
+    <col min="1" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Nova função no controller do candidateService
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="21">
   <si>
     <t>Mestrados</t>
   </si>
@@ -39,25 +39,28 @@
     <t>Nível</t>
   </si>
   <si>
+    <t>{"id":1,"editalPosition":1,"editalId":"001-2023","begin":null,"finish":null,"currentStep":0,"name":"test1","socialName":"test1name","address":null,"neighborhood":null,"city":null,"uf":null,"cep":null,"email":"test@email.com","birthday":null,"nationality":null,"country":null,"passport":null,"cpf":null,"gender":null,"homePhone":null,"cellPhone":null,"desiredCourse":"Eng","polity":null,"inscricaoposcomp":"Mestrado","anoposcomp":null,"notaposcomp":null,"solicitabolsa":null,"tituloproposta":null,"cartaorientador":"Dr. test","motivos":null,"proposta":null,"curriculum":null,"prova_anterior":null,"diploma":null,"cotas":null,"status":"0"}</t>
+  </si>
+  <si>
+    <t>{"id":2,"editalPosition":2,"editalId":"001-2023","begin":null,"finish":null,"currentStep":0,"name":"test2","socialName":"nameTest","address":null,"neighborhood":null,"city":null,"uf":null,"cep":null,"email":"aluno_test@email.com","birthday":null,"nationality":null,"country":null,"passport":null,"cpf":null,"gender":null,"homePhone":null,"cellPhone":null,"desiredCourse":"Eng","polity":null,"inscricaoposcomp":"Doutorado","anoposcomp":null,"notaposcomp":null,"solicitabolsa":null,"tituloproposta":null,"cartaorientador":"Dr. test","motivos":null,"proposta":null,"curriculum":null,"prova_anterior":null,"diploma":null,"cotas":null,"status":"0"}</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Doutorados</t>
+  </si>
+  <si>
+    <t>Teste2</t>
+  </si>
+  <si>
+    <t>asd@asd.com</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
     <t>Teste</t>
-  </si>
-  <si>
-    <t>asd@email.com</t>
-  </si>
-  <si>
-    <t>123456</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Doutorados</t>
-  </si>
-  <si>
-    <t>Teste2</t>
-  </si>
-  <si>
-    <t>asd@asd.com</t>
   </si>
   <si>
     <t>Nota Final</t>
@@ -513,37 +516,22 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -574,25 +562,25 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -625,15 +613,15 @@
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C3" s="1"/>
     </row>
@@ -645,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -677,24 +665,24 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -705,16 +693,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionado tabela de Titulos
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -7,13 +7,15 @@
     <sheet sheetId="1" name="Candidato" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Provas" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Propostas" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Titulos" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Média Final" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="42">
   <si>
     <t>Mestrados</t>
   </si>
@@ -39,28 +41,49 @@
     <t>Nível</t>
   </si>
   <si>
-    <t>{"id":1,"editalPosition":1,"editalId":"001-2023","begin":null,"finish":null,"currentStep":0,"name":"test1","socialName":"test1name","address":null,"neighborhood":null,"city":null,"uf":null,"cep":null,"email":"test@email.com","birthday":null,"nationality":null,"country":null,"passport":null,"cpf":null,"gender":null,"homePhone":null,"cellPhone":null,"desiredCourse":"Eng","polity":null,"inscricaoposcomp":"Mestrado","anoposcomp":null,"notaposcomp":null,"solicitabolsa":null,"tituloproposta":null,"cartaorientador":"Dr. test","motivos":null,"proposta":null,"curriculum":null,"prova_anterior":null,"diploma":null,"cotas":null,"status":"0"}</t>
-  </si>
-  <si>
-    <t>{"id":2,"editalPosition":2,"editalId":"001-2023","begin":null,"finish":null,"currentStep":0,"name":"test2","socialName":"nameTest","address":null,"neighborhood":null,"city":null,"uf":null,"cep":null,"email":"aluno_test@email.com","birthday":null,"nationality":null,"country":null,"passport":null,"cpf":null,"gender":null,"homePhone":null,"cellPhone":null,"desiredCourse":"Eng","polity":null,"inscricaoposcomp":"Doutorado","anoposcomp":null,"notaposcomp":null,"solicitabolsa":null,"tituloproposta":null,"cartaorientador":"Dr. test","motivos":null,"proposta":null,"curriculum":null,"prova_anterior":null,"diploma":null,"cotas":null,"status":"0"}</t>
-  </si>
-  <si>
-    <t/>
+    <t>Comprovante</t>
+  </si>
+  <si>
+    <t>Curriculum</t>
+  </si>
+  <si>
+    <t>Historico</t>
+  </si>
+  <si>
+    <t>Proposto</t>
+  </si>
+  <si>
+    <t>Cartas (2 no minimo)</t>
+  </si>
+  <si>
+    <t>Homologado</t>
+  </si>
+  <si>
+    <t>Observacoes</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test@email.com</t>
+  </si>
+  <si>
+    <t>completo</t>
+  </si>
+  <si>
+    <t>Mestrado</t>
   </si>
   <si>
     <t>Doutorados</t>
   </si>
   <si>
-    <t>Teste2</t>
-  </si>
-  <si>
-    <t>asd@asd.com</t>
-  </si>
-  <si>
-    <t>123456</t>
-  </si>
-  <si>
-    <t>Teste</t>
+    <t>test2</t>
+  </si>
+  <si>
+    <t>johonTest@email.com</t>
+  </si>
+  <si>
+    <t>Doutorado</t>
   </si>
   <si>
     <t>Nota Final</t>
@@ -76,6 +99,48 @@
   </si>
   <si>
     <t>Media Final</t>
+  </si>
+  <si>
+    <t>Atividades</t>
+  </si>
+  <si>
+    <t>Publicações</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>NAC</t>
+  </si>
+  <si>
+    <t>Estágio, Extensão e monitoria</t>
+  </si>
+  <si>
+    <t>Docência</t>
+  </si>
+  <si>
+    <t>IC, IT, ID</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B1 a B2</t>
+  </si>
+  <si>
+    <t>B3 a B5</t>
+  </si>
+  <si>
+    <t>Prova</t>
+  </si>
+  <si>
+    <t>Proposta</t>
+  </si>
+  <si>
+    <t>Títulos</t>
+  </si>
+  <si>
+    <t>Média</t>
   </si>
 </sst>
 </file>
@@ -91,6 +156,7 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
       <color rgb="FFFFFF"/>
     </font>
     <font>
@@ -124,14 +190,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,118 +543,165 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="7" width="15" customWidth="1"/>
+    <col min="6" max="11" width="15" customWidth="1"/>
+    <col min="12" max="14" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
+    <row r="1" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="2" t="s">
-        <v>0</v>
-      </c>
+      <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-    </row>
-    <row r="5" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="M5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A4:K4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -591,52 +709,70 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="3" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3">
+        <f>=Candidato!B:B</f>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
+      <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3">
+        <f>=Candidato!B:B</f>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -644,68 +780,378 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="str">
+        <f>SUM(B2:D2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <f>SUM(B2:D2)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="10" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3" t="str">
+        <f>=IF(SUM(B2:E2)&gt;30,30,SUM(B2:E2)) + IF(SUM(F2:H2)&gt;70,70,SUM(F2:H2))</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="str">
+        <f>=5+((5 * I2)/100)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="I8" s="3" t="str">
+        <f>=IF(SUM(B2:E2)&gt;30,30,SUM(B2:E2)) + IF(SUM(F2:H2)&gt;70,70,SUM(F2:H2))</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="str">
+        <f>=5+((5 * I2)/100)</f>
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="J6:J7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="5" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3">
+        <f>=Provas!C:C</f>
+      </c>
+      <c r="C3" s="3">
+        <f>=Propostas!E:E</f>
+      </c>
+      <c r="D3" s="3" t="str">
+        <f>=Titulos!I2</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="str">
+        <f>AVERAGE(B2:D2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="40" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="B5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="B6" s="3">
+        <f>=Provas!C:C</f>
+      </c>
+      <c r="C6" s="3">
+        <f>=Propostas!E:E</f>
+      </c>
+      <c r="D6" s="3" t="str">
+        <f>=Titulos!I2</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <f>AVERAGE(B2:D2)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>